<commit_message>
docs: align MindToDoc with system-design-doc and add migration samples
Retire HTML prototype workflow in favor of UI annotation and config-table
derived docs; archive 2026-06-01 superpowers specs; add World Cup
system-design-doc samples and updated test-config outputs.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/output/test-config/ActivitySoccerLanguage.xlsx
+++ b/output/test-config/ActivitySoccerLanguage.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C58"/>
+  <dimension ref="A1:C175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -448,7 +448,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CfgID</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -463,7 +463,11 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr"/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
       <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr"/>
     </row>
@@ -706,644 +710,2633 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ActvSoccer_preset_name_2</t>
+          <t>ActvSoccer_preset_name_5</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>中路任意球</t>
+          <t>左路单刀</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>SlicePresetCfg/2</t>
+          <t>SlicePresetCfg/5</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ActvSoccer_preset_name_3</t>
+          <t>ActvSoccer_preset_name_6</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>标准点球</t>
+          <t>中路突破</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>SlicePresetCfg/3</t>
+          <t>SlicePresetCfg/6</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ActvSoccer_preset_name_4</t>
+          <t>ActvSoccer_preset_name_16</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>基础守门</t>
+          <t>中路吊射</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>SlicePresetCfg/4</t>
+          <t>SlicePresetCfg/16</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ActvSoccer_growth_fame_title_1</t>
+          <t>ActvSoccer_preset_name_2</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>业余球员</t>
+          <t>中路任意球</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GrowthLevelCfg/101</t>
+          <t>SlicePresetCfg/2</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ActvSoccer_growth_fame_title_2</t>
+          <t>ActvSoccer_preset_name_7</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>专业球员</t>
+          <t>左侧任意球</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GrowthLevelCfg/102</t>
+          <t>SlicePresetCfg/7</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ActvSoccer_growth_fame_title_3</t>
+          <t>ActvSoccer_preset_name_8</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>大师</t>
+          <t>右侧任意球</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>GrowthLevelCfg/103</t>
+          <t>SlicePresetCfg/8</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ActvSoccer_team_name_101</t>
+          <t>ActvSoccer_preset_name_17</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>红星联</t>
+          <t>弧线任意球</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>TeamCfg/101</t>
+          <t>SlicePresetCfg/17</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ActvSoccer_team_name_102</t>
+          <t>ActvSoccer_preset_name_3</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>莱茵青年</t>
+          <t>标准点球</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>TeamCfg/102</t>
+          <t>SlicePresetCfg/3</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ActvSoccer_team_name_103</t>
+          <t>ActvSoccer_preset_name_9</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>桑巴之星</t>
+          <t>加压点球</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>TeamCfg/103</t>
+          <t>SlicePresetCfg/9</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ActvSoccer_team_name_104</t>
+          <t>ActvSoccer_preset_name_10</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>蓝白雄鹰</t>
+          <t>左角球</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>TeamCfg/104</t>
+          <t>SlicePresetCfg/10</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ActvSoccer_team_name_201</t>
+          <t>ActvSoccer_preset_name_11</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>海港FC</t>
+          <t>右角球</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>TeamCfg/201</t>
+          <t>SlicePresetCfg/11</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ActvSoccer_team_name_202</t>
+          <t>ActvSoccer_preset_name_18</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>东方之鹰</t>
+          <t>后点包抄</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>TeamCfg/202</t>
+          <t>SlicePresetCfg/18</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ActvSoccer_team_name_203</t>
+          <t>ActvSoccer_preset_name_12</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>北欧狼</t>
+          <t>左界外球</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>TeamCfg/203</t>
+          <t>SlicePresetCfg/12</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ActvSoccer_team_name_204</t>
+          <t>ActvSoccer_preset_name_13</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>阿根廷神鹰</t>
+          <t>右界外球</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>TeamCfg/204</t>
+          <t>SlicePresetCfg/13</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ActvSoccer_team_name_205</t>
+          <t>ActvSoccer_preset_name_4</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>桑巴红魔</t>
+          <t>基础守门</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>TeamCfg/205</t>
+          <t>SlicePresetCfg/4</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ActvSoccer_team_name_206</t>
+          <t>ActvSoccer_preset_name_14</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>南美风暴</t>
+          <t>大范围守门</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>TeamCfg/206</t>
+          <t>SlicePresetCfg/14</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ActvSoccer_team_name_207</t>
+          <t>ActvSoccer_preset_name_15</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>潘帕斯之翼</t>
+          <t>近距扑点</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>TeamCfg/207</t>
+          <t>SlicePresetCfg/15</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ActvSoccer_team_name_208</t>
+          <t>ActvSoccer_growth_fame_title_1</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>高卢雄鸡</t>
+          <t>业余球员</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>TeamCfg/208</t>
+          <t>FameGrowthLevelCfg/1</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ActvSoccer_season_league_name_1</t>
+          <t>ActvSoccer_growth_fame_title_2</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>地区预选赛</t>
+          <t>新秀</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>SeasonCfg/1</t>
+          <t>FameGrowthLevelCfg/2</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_phase_name_team_build</t>
+          <t>ActvSoccer_growth_fame_title_3</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>组队期</t>
+          <t>专业球员</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/1</t>
+          <t>FameGrowthLevelCfg/3</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_day_content_1</t>
+          <t>ActvSoccer_growth_fame_title_4</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>发起/加入组队、命名队名队标、审批</t>
+          <t>明星</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/1</t>
+          <t>FameGrowthLevelCfg/4</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_day_content_2</t>
+          <t>ActvSoccer_growth_fame_title_5</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>组队结束补位</t>
+          <t>大师</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/2</t>
+          <t>FameGrowthLevelCfg/5</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_phase_name_3</t>
+          <t>ActvSoccer_growth_fame_title_6</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>海选</t>
+          <t>世界级</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/3</t>
+          <t>FameGrowthLevelCfg/6</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_day_content_3</t>
+          <t>ActvSoccer_growth_fame_title_7</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>1天内筛出64强</t>
+          <t>传奇</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/3</t>
+          <t>FameGrowthLevelCfg/7</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_phase_name_4</t>
+          <t>ActvSoccer_team_name_101</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>正赛第1轮</t>
+          <t>红星联</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/4</t>
+          <t>TeamCfg/101</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_day_content_4</t>
+          <t>ActvSoccer_team_name_102</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>8组各一轮(64强)</t>
+          <t>莱茵青年</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/4</t>
+          <t>TeamCfg/102</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_phase_name_5</t>
+          <t>ActvSoccer_team_name_103</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>正赛第2轮</t>
+          <t>桑巴之星</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/5</t>
+          <t>TeamCfg/103</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_day_content_5</t>
+          <t>ActvSoccer_team_name_104</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>8组各一轮(32强)</t>
+          <t>蓝白雄鹰</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/5</t>
+          <t>TeamCfg/104</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_phase_name_6</t>
+          <t>ActvSoccer_team_name_201</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>正赛第3轮</t>
+          <t>海港FC</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/6</t>
+          <t>TeamCfg/201</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_day_content_6</t>
+          <t>ActvSoccer_team_name_202</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>8组各一轮(16强)</t>
+          <t>东方之鹰</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/6</t>
+          <t>TeamCfg/202</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_phase_name_7</t>
+          <t>ActvSoccer_team_name_203</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>正赛第4轮</t>
+          <t>北欧狼</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/7</t>
+          <t>TeamCfg/203</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_day_content_7</t>
+          <t>ActvSoccer_team_name_204</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>8组决出组冠军→8强</t>
+          <t>阿根廷神鹰</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/7</t>
+          <t>TeamCfg/204</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_phase_name_8</t>
+          <t>ActvSoccer_team_name_205</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>正赛第5轮</t>
+          <t>桑巴红魔</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/8</t>
+          <t>TeamCfg/205</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_day_content_8</t>
+          <t>ActvSoccer_team_name_206</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>8强淘汰赛(4强)</t>
+          <t>南美风暴</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/8</t>
+          <t>TeamCfg/206</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_phase_name_9</t>
+          <t>ActvSoccer_team_name_207</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>决赛</t>
+          <t>潘帕斯之翼</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/9</t>
+          <t>TeamCfg/207</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_day_content_9</t>
+          <t>ActvSoccer_team_name_208</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>冠亚军决赛</t>
+          <t>高卢雄鸡</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/9</t>
+          <t>TeamCfg/208</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ActvSoccer_knockout_phase_name_10</t>
+          <t>ActvSoccer_team_name_3001</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>展示期</t>
+          <t>社区杯·联</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>KnockoutPhaseCfg/10</t>
+          <t>TeamCfg/3001</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
+          <t>ActvSoccer_team_name_3002</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>社区杯·FC</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>TeamCfg/3002</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3003</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>社区杯·竞技</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>TeamCfg/3003</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3004</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>社区杯·联合</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>TeamCfg/3004</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3005</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>社区杯·勇士</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>TeamCfg/3005</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3006</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>城市联赛·联</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>TeamCfg/3006</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3007</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>城市联赛·FC</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>TeamCfg/3007</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3008</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>城市联赛·竞技</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>TeamCfg/3008</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3009</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>城市联赛·联合</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>TeamCfg/3009</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3010</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>城市联赛·勇士</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>TeamCfg/3010</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3011</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>省级联赛·联</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>TeamCfg/3011</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3012</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>省级联赛·FC</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>TeamCfg/3012</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3013</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>省级联赛·竞技</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>TeamCfg/3013</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3014</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>省级联赛·联合</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>TeamCfg/3014</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3015</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>省级联赛·勇士</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>TeamCfg/3015</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3016</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>大区联赛·联</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>TeamCfg/3016</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3017</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>大区联赛·FC</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>TeamCfg/3017</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3018</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>大区联赛·竞技</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>TeamCfg/3018</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3019</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>大区联赛·联合</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>TeamCfg/3019</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3020</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>大区联赛·勇士</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>TeamCfg/3020</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3021</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>全国联赛·联</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>TeamCfg/3021</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3022</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>全国联赛·FC</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>TeamCfg/3022</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3023</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>全国联赛·竞技</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>TeamCfg/3023</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3024</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>全国联赛·联合</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>TeamCfg/3024</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3025</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>全国联赛·勇士</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>TeamCfg/3025</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3026</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>洲际资格赛·联</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>TeamCfg/3026</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3027</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>洲际资格赛·FC</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>TeamCfg/3027</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3028</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>洲际资格赛·竞技</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>TeamCfg/3028</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3029</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>洲际资格赛·联合</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>TeamCfg/3029</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3030</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>洲际资格赛·勇士</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>TeamCfg/3030</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3031</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>洲际联赛·联</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>TeamCfg/3031</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3032</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>洲际联赛·FC</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>TeamCfg/3032</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3033</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>洲际联赛·竞技</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>TeamCfg/3033</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3034</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>洲际联赛·联合</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>TeamCfg/3034</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3035</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>洲际联赛·勇士</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>TeamCfg/3035</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3036</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>国际邀请赛·联</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>TeamCfg/3036</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3037</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>国际邀请赛·FC</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>TeamCfg/3037</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3038</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>国际邀请赛·竞技</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>TeamCfg/3038</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3039</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>国际邀请赛·联合</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>TeamCfg/3039</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3040</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>国际邀请赛·勇士</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>TeamCfg/3040</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3041</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>世界精英赛·联</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>TeamCfg/3041</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3042</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>世界精英赛·FC</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>TeamCfg/3042</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3043</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>世界精英赛·竞技</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>TeamCfg/3043</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3044</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>世界精英赛·联合</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>TeamCfg/3044</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3045</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>世界精英赛·勇士</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>TeamCfg/3045</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3046</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>世界杯总决赛·联</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>TeamCfg/3046</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3047</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>世界杯总决赛·FC</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>TeamCfg/3047</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3048</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>世界杯总决赛·竞技</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>TeamCfg/3048</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3049</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>世界杯总决赛·联合</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>TeamCfg/3049</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>ActvSoccer_team_name_3050</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>世界杯总决赛·勇士</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>TeamCfg/3050</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_1</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>社区杯 第1/50轮</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>SeasonCfg/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_2</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>社区杯 第2/50轮</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>SeasonCfg/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_3</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>社区杯 第3/50轮</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>SeasonCfg/3</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_4</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>社区杯 第4/50轮</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>SeasonCfg/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_5</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>社区杯 第5/50轮</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>SeasonCfg/5</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_6</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>城市联赛 第6/50轮</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>SeasonCfg/6</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_7</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>城市联赛 第7/50轮</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>SeasonCfg/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_8</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>城市联赛 第8/50轮</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>SeasonCfg/8</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_9</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>城市联赛 第9/50轮</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>SeasonCfg/9</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_10</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>城市联赛 第10/50轮</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>SeasonCfg/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_11</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>省级联赛 第11/50轮</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>SeasonCfg/11</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_12</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>省级联赛 第12/50轮</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>SeasonCfg/12</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_13</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>省级联赛 第13/50轮</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>SeasonCfg/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_14</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>省级联赛 第14/50轮</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>SeasonCfg/14</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_15</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>省级联赛 第15/50轮</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>SeasonCfg/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_16</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>大区联赛 第16/50轮</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>SeasonCfg/16</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_17</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>大区联赛 第17/50轮</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>SeasonCfg/17</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_18</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>大区联赛 第18/50轮</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>SeasonCfg/18</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_19</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>大区联赛 第19/50轮</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>SeasonCfg/19</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_20</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>大区联赛 第20/50轮</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>SeasonCfg/20</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_21</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>全国联赛 第21/50轮</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>SeasonCfg/21</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_22</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>全国联赛 第22/50轮</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>SeasonCfg/22</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_23</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>全国联赛 第23/50轮</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>SeasonCfg/23</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_24</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>全国联赛 第24/50轮</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>SeasonCfg/24</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_25</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>全国联赛 第25/50轮</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>SeasonCfg/25</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_26</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>洲际资格赛 第26/50轮</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>SeasonCfg/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_27</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>洲际资格赛 第27/50轮</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>SeasonCfg/27</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_28</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>洲际资格赛 第28/50轮</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>SeasonCfg/28</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_29</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>洲际资格赛 第29/50轮</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>SeasonCfg/29</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_30</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>洲际资格赛 第30/50轮</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>SeasonCfg/30</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_31</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>洲际联赛 第31/50轮</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>SeasonCfg/31</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_32</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>洲际联赛 第32/50轮</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>SeasonCfg/32</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_33</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>洲际联赛 第33/50轮</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>SeasonCfg/33</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_34</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>洲际联赛 第34/50轮</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>SeasonCfg/34</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_35</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>洲际联赛 第35/50轮</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>SeasonCfg/35</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_36</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>国际邀请赛 第36/50轮</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>SeasonCfg/36</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_37</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>国际邀请赛 第37/50轮</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>SeasonCfg/37</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_38</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>国际邀请赛 第38/50轮</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>SeasonCfg/38</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_39</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>国际邀请赛 第39/50轮</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>SeasonCfg/39</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_40</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>国际邀请赛 第40/50轮</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>SeasonCfg/40</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_41</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>世界精英赛 第41/50轮</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>SeasonCfg/41</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_42</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>世界精英赛 第42/50轮</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>SeasonCfg/42</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_43</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>世界精英赛 第43/50轮</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>SeasonCfg/43</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_44</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>世界精英赛 第44/50轮</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>SeasonCfg/44</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_45</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>世界精英赛 第45/50轮</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>SeasonCfg/45</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_46</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>世界杯总决赛 第46/50轮</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>SeasonCfg/46</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_47</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>世界杯总决赛 第47/50轮</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>SeasonCfg/47</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_48</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>世界杯总决赛 第48/50轮</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>SeasonCfg/48</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_49</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>世界杯总决赛 第49/50轮</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>SeasonCfg/49</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>ActvSoccer_season_league_name_50</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>世界杯总决赛 第50/50轮</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>SeasonCfg/50</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_phase_name_team_build</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>组队期</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_day_content_1</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>发起/加入组队、命名队名队标、审批</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/1</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_day_content_2</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>组队结束补位</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/2</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_phase_name_3</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>海选</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/3</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_day_content_3</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>1天内筛出64强</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/3</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_phase_name_4</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>正赛第1轮</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_day_content_4</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>8组各一轮(64强)</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_phase_name_5</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>正赛第2轮</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/5</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_day_content_5</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>8组各一轮(32强)</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/5</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_phase_name_6</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>正赛第3轮</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/6</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_day_content_6</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>8组各一轮(16强)</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/6</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_phase_name_7</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>正赛第4轮</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_day_content_7</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>8组决出组冠军→8强</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/7</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_phase_name_8</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>正赛第5轮</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/8</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_day_content_8</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>8强淘汰赛(4强)</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/8</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_phase_name_9</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>决赛</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/9</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_day_content_9</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>冠亚军决赛</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/9</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>ActvSoccer_knockout_phase_name_10</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>展示期</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>KnockoutPhaseCfg/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
           <t>ActvSoccer_knockout_day_content_10</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
+      <c r="B175" t="inlineStr">
         <is>
           <t>冠军展示+兑换商店可用</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C175" t="inlineStr">
         <is>
           <t>KnockoutPhaseCfg/10</t>
         </is>

</xml_diff>